<commit_message>
Optimization of main function
</commit_message>
<xml_diff>
--- a/backend/PS93_Customer.xlsx
+++ b/backend/PS93_Customer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LK627GW\Downloads\Data_Harmonization 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://people.ey.com/personal/nitish_t_gds_ey_com/Documents/Desktop/DataHEC/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE12DFD-1770-4C63-8B59-1FA2000709A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{BBE12DFD-1770-4C63-8B59-1FA2000709A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C11223F4-E94E-4192-94B1-2D9532C06D71}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="14400" windowHeight="8260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="15220" yWindow="6460" windowWidth="5000" windowHeight="4200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1255,6 +1255,9 @@
   <dimension ref="A1:O30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.08984375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.08984375" customWidth="1"/>
     <col min="12" max="12" width="14.1796875" customWidth="1"/>
     <col min="15" max="15" width="18.7265625" customWidth="1"/>

</xml_diff>